<commit_message>
Update header-dark and sidebar-monogram templates, PDF helpers, and miscellaneous file changes
</commit_message>
<xml_diff>
--- a/seo/Keywords medium.xlsx
+++ b/seo/Keywords medium.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/elw/Documents/Test/AI/AI-Resume-Builder/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/elw/Documents/Test/AI/AI-Resume-Builder/seo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63378436-F593-274A-8F29-05716710286A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4215B290-9BAC-414B-8F03-3A1B418EA6E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="300" yWindow="2700" windowWidth="35120" windowHeight="16940" xr2:uid="{8BE718A7-387B-A84F-85B5-D1553FCC480A}"/>
   </bookViews>
@@ -763,15 +763,15 @@
     <col min="2" max="3" width="25" customWidth="1"/>
     <col min="4" max="4" width="24.5" customWidth="1"/>
     <col min="5" max="5" width="25" customWidth="1"/>
-    <col min="6" max="6" width="25.33203125" customWidth="1"/>
+    <col min="6" max="6" width="29.5" customWidth="1"/>
     <col min="7" max="7" width="20.5" customWidth="1"/>
     <col min="8" max="8" width="23.1640625" customWidth="1"/>
     <col min="9" max="9" width="21.6640625" customWidth="1"/>
     <col min="10" max="10" width="17.83203125" customWidth="1"/>
-    <col min="11" max="11" width="16.6640625" customWidth="1"/>
-    <col min="12" max="12" width="17.33203125" customWidth="1"/>
-    <col min="13" max="13" width="18.5" customWidth="1"/>
-    <col min="14" max="14" width="15" customWidth="1"/>
+    <col min="11" max="11" width="21" customWidth="1"/>
+    <col min="12" max="12" width="24" customWidth="1"/>
+    <col min="13" max="13" width="26.33203125" customWidth="1"/>
+    <col min="14" max="14" width="24.83203125" customWidth="1"/>
     <col min="15" max="15" width="18.6640625" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>